<commit_message>
timeslots added for manual schedules
</commit_message>
<xml_diff>
--- a/data/B24_department_schedules_finals/Bilgisayar Mühendisliği.xlsx
+++ b/data/B24_department_schedules_finals/Bilgisayar Mühendisliği.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\B24_department_schedules_finals\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e402f802124af4b/Masaüstü/Projects/Campus-Scheduling/data/B24_department_schedules_finals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A411358-8EB3-4463-B267-6244C2178277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{4A411358-8EB3-4463-B267-6244C2178277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFEADF54-3619-4E6C-B3C5-DBAACF684721}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20760" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -283,7 +283,7 @@
     <t>Amfi 3</t>
   </si>
   <si>
-    <t>Timeslot</t>
+    <t>timeslots</t>
   </si>
 </sst>
 </file>
@@ -480,7 +480,7 @@
     <tableColumn id="4" xr3:uid="{B34557C0-D930-44D9-A811-D5F01B299ECF}" name="Rooms" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{C09534FA-04D2-48E5-8497-0DB03EB02FC5}" name="Course Name" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{C7781146-3CF4-4B66-B0B2-F7C86896AE17}" name="Rooms Used" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{1EF90761-711D-44B5-A423-74A2E99CD9EE}" name="Timeslot" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{1EF90761-711D-44B5-A423-74A2E99CD9EE}" name="timeslots" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium22" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -774,14 +774,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="10.90625" customWidth="1"/>
-    <col min="5" max="5" width="35.26953125" customWidth="1"/>
-    <col min="6" max="6" width="56.36328125" customWidth="1"/>
+    <col min="2" max="2" width="10.9296875" customWidth="1"/>
+    <col min="5" max="5" width="35.265625" customWidth="1"/>
+    <col min="6" max="6" width="56.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -804,7 +804,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -827,7 +827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -850,7 +850,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -874,7 +874,7 @@
       </c>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -898,7 +898,7 @@
       </c>
       <c r="J5" s="7"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>1</v>
       </c>
@@ -922,7 +922,7 @@
       </c>
       <c r="J6" s="7"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>1</v>
       </c>
@@ -947,7 +947,7 @@
       <c r="J7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>1</v>
       </c>
@@ -972,7 +972,7 @@
       <c r="J8" s="7"/>
       <c r="M8" s="7"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>1</v>
       </c>
@@ -997,7 +997,7 @@
       <c r="J9" s="7"/>
       <c r="M9" s="7"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="3">
         <v>2</v>
       </c>
@@ -1022,7 +1022,7 @@
       <c r="J10" s="7"/>
       <c r="M10" s="7"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="3">
         <v>2</v>
       </c>
@@ -1047,7 +1047,7 @@
       <c r="J11" s="7"/>
       <c r="M11" s="7"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -1072,7 +1072,7 @@
       <c r="J12" s="7"/>
       <c r="M12" s="7"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="3">
         <v>2</v>
       </c>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="M13" s="7"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="3">
         <v>2</v>
       </c>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="M14" s="7"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="4">
         <v>3</v>
       </c>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="M15" s="7"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="4">
         <v>3</v>
       </c>
@@ -1167,7 +1167,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="4">
         <v>3</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="4">
         <v>3</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="4">
         <v>3</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" s="4">
         <v>3</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4">
         <v>3</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="4">
         <v>3</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="4">
         <v>3</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="5">
         <v>4</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="5">
         <v>4</v>
       </c>
@@ -1374,7 +1374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="5">
         <v>4</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="5">
         <v>4</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="5">
         <v>4</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="5">
         <v>4</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="5">
         <v>4</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="5">
         <v>4</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="5">
         <v>4</v>
       </c>

</xml_diff>